<commit_message>
Wprowadzono cennik oraz panel administratora (nietestowyny)
</commit_message>
<xml_diff>
--- a/backend/data/price_catalog.xlsx
+++ b/backend/data/price_catalog.xlsx
@@ -495,7 +495,9 @@
           <t>m³</t>
         </is>
       </c>
-      <c r="C2" s="3" t="n"/>
+      <c r="C2" s="3" t="n">
+        <v>2450</v>
+      </c>
       <c r="D2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
@@ -509,7 +511,9 @@
           <t>szt</t>
         </is>
       </c>
-      <c r="C3" s="3" t="n"/>
+      <c r="C3" s="3" t="n">
+        <v>1200</v>
+      </c>
       <c r="D3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
@@ -1293,7 +1297,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -1406,47 +1410,54 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>5. Jeśli plik jest otwarty w Excelu w momencie liczenia przedmiaru w aplikacji,</t>
+          <t>5. Po edycji zapisz plik i wgraj go z powrotem przyciskiem 'Wgraj cennik' w aplikacji</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t xml:space="preserve">   automatyczne dopisanie nowych pozycji zostanie pominięte (Windows blokuje</t>
+          <t xml:space="preserve">   (przycisk 'Pobierz cennik' służy do pobrania aktualnej wersji do edycji).</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t xml:space="preserve">   zapis do otwartego pliku) — zamknij plik, aby nowe pozycje mogły się dopisać.</t>
+          <t xml:space="preserve">   Wgranie scala Twoje zmiany z serwerem — pozycje dopisane w międzyczasie przez</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>6. Nie zostawiaj pustych wierszy pomiędzy danymi w arkuszu 'Ceny' — pusty</t>
+          <t xml:space="preserve">   innych użytkowników nie zostaną skasowane.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t xml:space="preserve">   'Opis pozycji' kończy odczyt arkusza.</t>
+          <t>6. Nie zostawiaj pustych wierszy pomiędzy danymi w arkuszu 'Ceny' — pusty</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>7. Ceny są NETTO, w PLN — sposób ich interpretacji (netto/brutto) ustala użytkownik</t>
+          <t xml:space="preserve">   'Opis pozycji' kończy odczyt arkusza.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
+        <is>
+          <t>7. Ceny są NETTO, w PLN — sposób ich interpretacji (netto/brutto) ustala użytkownik</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
         <is>
           <t xml:space="preserve">   przy analizie wyniku przedmiaru.</t>
         </is>

</xml_diff>